<commit_message>
feat: Upload charge files to Azure and save them in the db (MPT-8992, MPT-8994)
</commit_message>
<xml_diff>
--- a/tests/commands/snapshots/test_generate_monthtly_charges/test_export_to_zip/charges_file.xlsx
+++ b/tests/commands/snapshots/test_generate_monthtly_charges/test_export_to_zip/charges_file.xlsx
@@ -61,7 +61,7 @@
     <t>subscription.externalIds.vendor</t>
   </si>
   <si>
-    <t>FORG-2846-5181-3940</t>
+    <t>FORG-7330-1645-9608</t>
   </si>
   <si>
     <t>item.externalIds.vendor</t>
@@ -88,7 +88,7 @@
     <t>-0.65</t>
   </si>
   <si>
-    <t>9a1de644-815e-46d1-bb8f-aa1837f8a88b</t>
+    <t>06cb0fb3-9a1d-4644-815e-f6d13b8faa18</t>
   </si>
   <si>
     <t>AWS Account</t>
@@ -97,10 +97,10 @@
     <t>GCP Account</t>
   </si>
   <si>
-    <t>b74d0fb1-32e7-4629-8fad-c1a606cb0fb3</t>
-  </si>
-  <si>
-    <t>6b65a6a4-8b81-48f6-b38a-088ca65ed389</t>
+    <t>a65ed389-b74d-4fb1-b2e7-06298fadc1a6</t>
+  </si>
+  <si>
+    <t>386ecbe0-6b65-46a4-8b81-48f6b38a088c</t>
   </si>
 </sst>
 </file>

</xml_diff>